<commit_message>
remove unnecessary .gitignore entries and add new Excel files for data analysis
</commit_message>
<xml_diff>
--- a/Result_Excel_file/Result.xlsx
+++ b/Result_Excel_file/Result.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\class\Xcel_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VISHWAS SHARMA\Documents\Xcel_portfolio\Result_Excel_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1376789B-5D7C-4419-954E-1EB1C7AC5CB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C8414E2-0FE4-4C4D-8DE9-EABB25E5E7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{05FF70D9-F110-4AC7-B864-5F51B176B318}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{05FF70D9-F110-4AC7-B864-5F51B176B318}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1843,7 +1843,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="StudentPhoto" spid="_x0000_s2126"/>
+                  <a14:cameraTool cellRange="StudentPhoto" spid="_x0000_s2138"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2052,13 +2052,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="StudentPhoto" spid="_x0000_s2127"/>
+                  <a14:cameraTool cellRange="StudentPhoto" spid="_x0000_s2139"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -2098,10 +2098,6 @@
     <mc:Fallback/>
   </mc:AlternateContent>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3012,7 +3008,7 @@
       </c>
       <c r="C6" s="33">
         <f>J34</f>
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D6" s="30"/>
       <c r="E6" s="82"/>
@@ -3034,7 +3030,7 @@
       </c>
       <c r="C7" s="34" t="str">
         <f>VLOOKUP(C6,Sheet1!B4:K14,MATCH(B7,Sheet1!B4:M4,0),0)</f>
-        <v>Jatin Tiwari</v>
+        <v>Vishwas Sharma</v>
       </c>
       <c r="D7" s="30"/>
       <c r="E7" s="82"/>
@@ -3056,7 +3052,7 @@
       </c>
       <c r="C8" s="34" t="str">
         <f>VLOOKUP(C6,Sheet1!B4:K14,MATCH(B8,Sheet1!B4:M4,0),0)</f>
-        <v>Hariom Tiwari</v>
+        <v>Yogesh Sharma</v>
       </c>
       <c r="D8" s="30"/>
       <c r="E8" s="82"/>
@@ -3077,7 +3073,7 @@
       </c>
       <c r="C9" s="34" t="str">
         <f>VLOOKUP(C6,Sheet1!B4:K14,MATCH(B9,Sheet1!B4:M4,0),0)</f>
-        <v>Jaya Tiwari</v>
+        <v>Sunanda Sharma</v>
       </c>
       <c r="D9" s="30"/>
       <c r="E9" s="82"/>
@@ -3119,7 +3115,7 @@
       </c>
       <c r="C11" s="35">
         <f>VLOOKUP(C6,Sheet1!B4:K14,MATCH(B11,Sheet1!B4:M4,0),0)</f>
-        <v>40651</v>
+        <v>40772</v>
       </c>
       <c r="D11" s="30"/>
       <c r="E11" s="82"/>
@@ -3227,14 +3223,14 @@
       </c>
       <c r="D16" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B16,Sheet1!B4:M4,0),0)</f>
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="E16" s="37">
         <v>35</v>
       </c>
       <c r="F16" s="38" t="str">
         <f t="shared" ref="F16:F21" si="0">IF(D16&gt;=E16,"PASS","FAIL")</f>
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="7"/>
@@ -3256,14 +3252,14 @@
       </c>
       <c r="D17" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B17,Sheet1!B4:M4,0),0)</f>
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="E17" s="37">
         <v>35</v>
       </c>
       <c r="F17" s="38" t="str">
         <f t="shared" si="0"/>
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="7"/>
@@ -3285,14 +3281,14 @@
       </c>
       <c r="D18" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B18,Sheet1!B4:M4,0),0)</f>
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="E18" s="37">
         <v>35</v>
       </c>
       <c r="F18" s="38" t="str">
         <f t="shared" si="0"/>
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="7"/>
@@ -3313,14 +3309,14 @@
       </c>
       <c r="D19" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B19,Sheet1!B4:M4,0),0)</f>
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="E19" s="37">
         <v>35</v>
       </c>
       <c r="F19" s="38" t="str">
         <f t="shared" si="0"/>
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="G19" s="5"/>
       <c r="H19" s="7"/>
@@ -3342,14 +3338,14 @@
       </c>
       <c r="D20" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B20,Sheet1!B4:M4,0),0)</f>
-        <v>18</v>
+        <v>83</v>
       </c>
       <c r="E20" s="37">
         <v>35</v>
       </c>
       <c r="F20" s="38" t="str">
         <f t="shared" si="0"/>
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="G20" s="5"/>
       <c r="H20" s="7"/>
@@ -3371,7 +3367,7 @@
       </c>
       <c r="D21" s="39">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B21,Sheet1!B4:M4,0),0)</f>
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="E21" s="39">
         <v>35</v>
@@ -3436,7 +3432,7 @@
       </c>
       <c r="C24" s="44" t="str">
         <f>IF(COUNTIF(F16:F21,"PASS")&gt;=4,"PASS","FAIL")</f>
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="D24" s="30"/>
       <c r="E24" s="63" t="s">
@@ -3444,7 +3440,7 @@
       </c>
       <c r="F24" s="38">
         <f>SUM(D16:D21)</f>
-        <v>143</v>
+        <v>387</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
@@ -3463,7 +3459,7 @@
       </c>
       <c r="C25" s="45" t="str" cm="1">
         <f t="array" ref="C25">_xlfn.IFS(F25&gt;=80%,"A",F25&gt;=60%,"B",F25&gt;=40%,"C",F25&lt;40%,"D")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="D25" s="30"/>
       <c r="E25" s="64" t="s">
@@ -3471,7 +3467,7 @@
       </c>
       <c r="F25" s="46">
         <f>AVERAGE(D16:D21)/100</f>
-        <v>0.23833333333333331</v>
+        <v>0.64500000000000002</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -3526,7 +3522,7 @@
       </c>
       <c r="C31" s="65">
         <f ca="1">TODAY()</f>
-        <v>46246</v>
+        <v>46259</v>
       </c>
       <c r="D31" s="54"/>
       <c r="E31" s="55" t="s">
@@ -3541,7 +3537,7 @@
         <v>62</v>
       </c>
       <c r="J34" s="80">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update cafe sales dashboard and result Excel file
</commit_message>
<xml_diff>
--- a/Result_Excel_file/Result.xlsx
+++ b/Result_Excel_file/Result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VISHWAS SHARMA\Documents\Xcel_portfolio\Result_Excel_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C8414E2-0FE4-4C4D-8DE9-EABB25E5E7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E7B028-A8D1-4235-97BF-6142FB2A5A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{05FF70D9-F110-4AC7-B864-5F51B176B318}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{05FF70D9-F110-4AC7-B864-5F51B176B318}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
   <si>
     <t>Roll No.</t>
   </si>
@@ -246,9 +246,6 @@
   </si>
   <si>
     <t xml:space="preserve">                       SECONDARY SCHOOL EXAMINATION,2026</t>
-  </si>
-  <si>
-    <t>Enter the Roll NO. of Student:</t>
   </si>
 </sst>
 </file>
@@ -920,7 +917,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1090,14 +1087,15 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1843,7 +1841,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="StudentPhoto" spid="_x0000_s2138"/>
+                  <a14:cameraTool cellRange="StudentPhoto" spid="_x0000_s2144"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2052,7 +2050,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="StudentPhoto" spid="_x0000_s2139"/>
+                  <a14:cameraTool cellRange="StudentPhoto" spid="_x0000_s2145"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3007,11 +3005,10 @@
         <v>37</v>
       </c>
       <c r="C6" s="33">
-        <f>J34</f>
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D6" s="30"/>
-      <c r="E6" s="82"/>
+      <c r="E6" s="80"/>
       <c r="F6" s="30"/>
       <c r="G6" s="5"/>
       <c r="H6" s="7"/>
@@ -3030,10 +3027,10 @@
       </c>
       <c r="C7" s="34" t="str">
         <f>VLOOKUP(C6,Sheet1!B4:K14,MATCH(B7,Sheet1!B4:M4,0),0)</f>
-        <v>Vishwas Sharma</v>
+        <v>Jatin Tiwari</v>
       </c>
       <c r="D7" s="30"/>
-      <c r="E7" s="82"/>
+      <c r="E7" s="80"/>
       <c r="F7" s="30"/>
       <c r="G7" s="5"/>
       <c r="H7" s="7"/>
@@ -3052,10 +3049,10 @@
       </c>
       <c r="C8" s="34" t="str">
         <f>VLOOKUP(C6,Sheet1!B4:K14,MATCH(B8,Sheet1!B4:M4,0),0)</f>
-        <v>Yogesh Sharma</v>
+        <v>Hariom Tiwari</v>
       </c>
       <c r="D8" s="30"/>
-      <c r="E8" s="82"/>
+      <c r="E8" s="80"/>
       <c r="F8" s="30"/>
       <c r="G8" s="5"/>
       <c r="H8" s="7"/>
@@ -3073,10 +3070,10 @@
       </c>
       <c r="C9" s="34" t="str">
         <f>VLOOKUP(C6,Sheet1!B4:K14,MATCH(B9,Sheet1!B4:M4,0),0)</f>
-        <v>Sunanda Sharma</v>
+        <v>Jaya Tiwari</v>
       </c>
       <c r="D9" s="30"/>
-      <c r="E9" s="82"/>
+      <c r="E9" s="80"/>
       <c r="F9" s="30"/>
       <c r="G9" s="5"/>
       <c r="H9" s="7"/>
@@ -3097,7 +3094,7 @@
         <v>59</v>
       </c>
       <c r="D10" s="30"/>
-      <c r="E10" s="82"/>
+      <c r="E10" s="80"/>
       <c r="F10" s="30"/>
       <c r="G10" s="5"/>
       <c r="H10" s="7"/>
@@ -3115,10 +3112,10 @@
       </c>
       <c r="C11" s="35">
         <f>VLOOKUP(C6,Sheet1!B4:K14,MATCH(B11,Sheet1!B4:M4,0),0)</f>
-        <v>40772</v>
+        <v>40651</v>
       </c>
       <c r="D11" s="30"/>
-      <c r="E11" s="82"/>
+      <c r="E11" s="80"/>
       <c r="F11" s="30"/>
       <c r="G11" s="5"/>
       <c r="H11" s="7"/>
@@ -3140,7 +3137,7 @@
         <v>PRAGATI CONVENT HIGHER SECONDARY SCHOOL</v>
       </c>
       <c r="D12" s="30"/>
-      <c r="E12" s="82"/>
+      <c r="E12" s="80"/>
       <c r="F12" s="30"/>
       <c r="G12" s="5"/>
       <c r="H12" s="7"/>
@@ -3223,14 +3220,14 @@
       </c>
       <c r="D16" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B16,Sheet1!B4:M4,0),0)</f>
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E16" s="37">
         <v>35</v>
       </c>
       <c r="F16" s="38" t="str">
         <f t="shared" ref="F16:F21" si="0">IF(D16&gt;=E16,"PASS","FAIL")</f>
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="7"/>
@@ -3252,14 +3249,14 @@
       </c>
       <c r="D17" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B17,Sheet1!B4:M4,0),0)</f>
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="E17" s="37">
         <v>35</v>
       </c>
       <c r="F17" s="38" t="str">
         <f t="shared" si="0"/>
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="7"/>
@@ -3281,14 +3278,14 @@
       </c>
       <c r="D18" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B18,Sheet1!B4:M4,0),0)</f>
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="E18" s="37">
         <v>35</v>
       </c>
       <c r="F18" s="38" t="str">
         <f t="shared" si="0"/>
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="7"/>
@@ -3309,14 +3306,14 @@
       </c>
       <c r="D19" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B19,Sheet1!B4:M4,0),0)</f>
-        <v>93</v>
+        <v>16</v>
       </c>
       <c r="E19" s="37">
         <v>35</v>
       </c>
       <c r="F19" s="38" t="str">
         <f t="shared" si="0"/>
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G19" s="5"/>
       <c r="H19" s="7"/>
@@ -3338,14 +3335,14 @@
       </c>
       <c r="D20" s="37">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B20,Sheet1!B4:M4,0),0)</f>
-        <v>83</v>
+        <v>18</v>
       </c>
       <c r="E20" s="37">
         <v>35</v>
       </c>
       <c r="F20" s="38" t="str">
         <f t="shared" si="0"/>
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="G20" s="5"/>
       <c r="H20" s="7"/>
@@ -3367,7 +3364,7 @@
       </c>
       <c r="D21" s="39">
         <f>VLOOKUP(C6,Sheet1!B4:M14,MATCH(Sheet2!B21,Sheet1!B4:M4,0),0)</f>
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="E21" s="39">
         <v>35</v>
@@ -3432,7 +3429,7 @@
       </c>
       <c r="C24" s="44" t="str">
         <f>IF(COUNTIF(F16:F21,"PASS")&gt;=4,"PASS","FAIL")</f>
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="D24" s="30"/>
       <c r="E24" s="63" t="s">
@@ -3440,7 +3437,7 @@
       </c>
       <c r="F24" s="38">
         <f>SUM(D16:D21)</f>
-        <v>387</v>
+        <v>143</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="7"/>
@@ -3459,7 +3456,7 @@
       </c>
       <c r="C25" s="45" t="str" cm="1">
         <f t="array" ref="C25">_xlfn.IFS(F25&gt;=80%,"A",F25&gt;=60%,"B",F25&gt;=40%,"C",F25&lt;40%,"D")</f>
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="D25" s="30"/>
       <c r="E25" s="64" t="s">
@@ -3467,7 +3464,7 @@
       </c>
       <c r="F25" s="46">
         <f>AVERAGE(D16:D21)/100</f>
-        <v>0.64500000000000002</v>
+        <v>0.23833333333333331</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -3505,8 +3502,8 @@
       <c r="D29" s="32"/>
       <c r="E29" s="32"/>
       <c r="F29" s="48"/>
-      <c r="J29" s="81"/>
-      <c r="K29" s="81"/>
+      <c r="J29" s="79"/>
+      <c r="K29" s="79"/>
     </row>
     <row r="30" spans="2:17" ht="75" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B30" s="50"/>
@@ -3522,7 +3519,7 @@
       </c>
       <c r="C31" s="65">
         <f ca="1">TODAY()</f>
-        <v>46259</v>
+        <v>46268</v>
       </c>
       <c r="D31" s="54"/>
       <c r="E31" s="55" t="s">
@@ -3531,14 +3528,10 @@
       <c r="F31" s="56"/>
     </row>
     <row r="32" spans="2:17" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="33" spans="9:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="34" spans="9:10" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="I34" s="79" t="s">
-        <v>62</v>
-      </c>
-      <c r="J34" s="80">
-        <v>101</v>
-      </c>
+    <row r="34" spans="9:11" ht="46" x14ac:dyDescent="1">
+      <c r="I34" s="81"/>
+      <c r="J34" s="82"/>
+      <c r="K34" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>